<commit_message>
Support variable EEM grids and smooth example plots
</commit_message>
<xml_diff>
--- a/examples/expected/黑_五区积分.xlsx
+++ b/examples/expected/黑_五区积分.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sheet1：列 Ex=200–500 nm/10；行 Em=250–600 nm/2</t>
+          <t>Sheet1 或首个工作表：首行 Ex、首列 Em；单调数值波长轴，可使用不同网格点数和间隔</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>插值矩阵中负数及 Em≤Ex 对积分记 0；各区二维梯形积分，边半权，角四分之一权</t>
+          <t>负数及 Em≤Ex 记 0；原仪器网格沿用二维梯形法，其他网格以三角网格线性插值并按边界裁剪积分</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PhiN_i=Phi_i×(73750/区域面积_i)；P_i=PhiN_i/sum(PhiN_i)</t>
+          <t>PhiN_i=Phi_i×(本文件各区域总面积/本文件区域面积_i)；P_i=PhiN_i/sum(PhiN_i)</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>插值点是估计值，输出矩阵适合绘图；定量结果与早先零值掩膜积分不可混用</t>
+          <t>插值点是估计值；不同扫描范围的 FRI 比例不可直接比较，应先统一波长范围</t>
         </is>
       </c>
     </row>
@@ -746,21 +746,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>文件名</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>区域</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>面积_nm2</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
@@ -769,65 +774,90 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>黑.xlsx</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>I</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="C2" t="n">
         <v>4000</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>18.4375</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>黑.xlsx</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>II</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="C3" t="n">
         <v>2500</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>29.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>黑.xlsx</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>III</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="C4" t="n">
         <v>11000</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>6.704545454545454</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>黑.xlsx</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>IV</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="C5" t="n">
         <v>8450</v>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>8.727810650887575</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>黑.xlsx</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>V</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="C6" t="n">
         <v>47800</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>1.542887029288703</v>
       </c>
     </row>

</xml_diff>